<commit_message>
Clarify Feishu field types: Upvote=Number, Launch_tags=Multi-select, URL fields=URL
</commit_message>
<xml_diff>
--- a/assets/feishu_bitable_template.xlsx
+++ b/assets/feishu_bitable_template.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[Text]</t>
+          <t>[Multi-select]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -638,12 +638,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Weekly upvote count</t>
+          <t>Weekly upvote count — set as Number type in Feishu</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Category tags (AI, Productivity, …)</t>
+          <t>Category tags (AI, Productivity, …) — set as Multi-select in Feishu</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -653,12 +653,12 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Product Hunt product URL</t>
+          <t>Product Hunt product URL — set as URL type in Feishu</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t>PH discussion thread link</t>
+          <t>PH discussion thread link — set as URL type in Feishu</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
@@ -668,7 +668,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Official website URL</t>
+          <t>Official website URL — set as URL type in Feishu</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">

</xml_diff>